<commit_message>
Phase 3: stage 05 attritional model and aggregate stop loss
Attritional cost per life (FGU trend, new ATTRITIONAL completion side, CoV floor, lognormal/normal by
Box-Muller on new MINSTD streams) + simulated large claims above t_sl; net claims budget; stop loss on
PCT_BUDGET/PCT_EPI/AMOUNT, gross or net of the programme PP option; structure quantiles for Exhibits
C1/C2; exposed lives. Exact match to a numpy oracle in line and claimant mode. Stage 04 stages
sim_gross/sim_iterations; 01b writes an empty int_members; simulator Cos.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UTL5cPxKguFWxKSpgQZCbz
</commit_message>
<xml_diff>
--- a/data/synthetic/XoL_Control_synthetic.xlsx
+++ b/data/synthetic/XoL_Control_synthetic.xlsx
@@ -1200,7 +1200,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G45"/>
+  <dimension ref="A1:G46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2271,7 +2271,7 @@
       <c r="E41" s="5" t="inlineStr"/>
       <c r="F41" s="5" t="inlineStr">
         <is>
-          <t>Stop loss: minimum CoV of the attritional loss ratio [required]</t>
+          <t>Stop loss: minimum CoV of the attritional cost per life [required]</t>
         </is>
       </c>
       <c r="G41" s="6" t="n"/>
@@ -2279,24 +2279,28 @@
     <row r="42">
       <c r="A42" s="5" t="inlineStr">
         <is>
-          <t>net_claims_budget</t>
+          <t>sl_attritional_dist</t>
         </is>
       </c>
       <c r="B42" s="5" t="inlineStr">
         <is>
-          <t>Cedant impact</t>
-        </is>
-      </c>
-      <c r="C42" s="6" t="n"/>
-      <c r="D42" s="5" t="inlineStr">
-        <is>
-          <t>quote ccy</t>
-        </is>
-      </c>
-      <c r="E42" s="5" t="inlineStr"/>
+          <t>Stochastic</t>
+        </is>
+      </c>
+      <c r="C42" s="6" t="inlineStr">
+        <is>
+          <t>LOGNORMAL</t>
+        </is>
+      </c>
+      <c r="D42" s="5" t="inlineStr"/>
+      <c r="E42" s="5" t="inlineStr">
+        <is>
+          <t>LOGNORMAL,NORMAL</t>
+        </is>
+      </c>
       <c r="F42" s="5" t="inlineStr">
         <is>
-          <t>Blank = best-estimate gross claims</t>
+          <t>Stop loss: distribution of the attritional cost per life [required]</t>
         </is>
       </c>
       <c r="G42" s="6" t="n"/>
@@ -2304,7 +2308,7 @@
     <row r="43">
       <c r="A43" s="5" t="inlineStr">
         <is>
-          <t>reference_lives</t>
+          <t>net_claims_budget</t>
         </is>
       </c>
       <c r="B43" s="5" t="inlineStr">
@@ -2312,16 +2316,16 @@
           <t>Cedant impact</t>
         </is>
       </c>
-      <c r="C43" s="6" t="inlineStr"/>
+      <c r="C43" s="6" t="n"/>
       <c r="D43" s="5" t="inlineStr">
         <is>
-          <t>lives</t>
+          <t>quote ccy</t>
         </is>
       </c>
       <c r="E43" s="5" t="inlineStr"/>
       <c r="F43" s="5" t="inlineStr">
         <is>
-          <t>Blank = expected lives for the quote year</t>
+          <t>Blank = best-estimate gross claims</t>
         </is>
       </c>
       <c r="G43" s="6" t="n"/>
@@ -2329,7 +2333,7 @@
     <row r="44">
       <c r="A44" s="5" t="inlineStr">
         <is>
-          <t>return_periods</t>
+          <t>reference_lives</t>
         </is>
       </c>
       <c r="B44" s="5" t="inlineStr">
@@ -2337,20 +2341,16 @@
           <t>Cedant impact</t>
         </is>
       </c>
-      <c r="C44" s="6" t="inlineStr">
-        <is>
-          <t>5,50,250</t>
-        </is>
-      </c>
+      <c r="C44" s="6" t="inlineStr"/>
       <c r="D44" s="5" t="inlineStr">
         <is>
-          <t>years</t>
+          <t>lives</t>
         </is>
       </c>
       <c r="E44" s="5" t="inlineStr"/>
       <c r="F44" s="5" t="inlineStr">
         <is>
-          <t>Return periods shown in Exhibit C2 [required]</t>
+          <t>Blank = expected lives for the quote year</t>
         </is>
       </c>
       <c r="G44" s="6" t="n"/>
@@ -2358,37 +2358,66 @@
     <row r="45">
       <c r="A45" s="5" t="inlineStr">
         <is>
+          <t>return_periods</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="inlineStr">
+        <is>
+          <t>Cedant impact</t>
+        </is>
+      </c>
+      <c r="C45" s="6" t="inlineStr">
+        <is>
+          <t>5,50,250</t>
+        </is>
+      </c>
+      <c r="D45" s="5" t="inlineStr">
+        <is>
+          <t>years</t>
+        </is>
+      </c>
+      <c r="E45" s="5" t="inlineStr"/>
+      <c r="F45" s="5" t="inlineStr">
+        <is>
+          <t>Return periods shown in Exhibit C2 [required]</t>
+        </is>
+      </c>
+      <c r="G45" s="6" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
           <t>currency_display</t>
         </is>
       </c>
-      <c r="B45" s="5" t="inlineStr">
+      <c r="B46" s="5" t="inlineStr">
         <is>
           <t>Cedant impact</t>
         </is>
       </c>
-      <c r="C45" s="6" t="inlineStr">
+      <c r="C46" s="6" t="inlineStr">
         <is>
           <t>QUOTE</t>
         </is>
       </c>
-      <c r="D45" s="5" t="inlineStr"/>
-      <c r="E45" s="5" t="inlineStr">
+      <c r="D46" s="5" t="inlineStr"/>
+      <c r="E46" s="5" t="inlineStr">
         <is>
           <t>QUOTE,USD</t>
         </is>
       </c>
-      <c r="F45" s="5" t="inlineStr">
+      <c r="F46" s="5" t="inlineStr">
         <is>
           <t>Currency of the client exhibits [required]</t>
         </is>
       </c>
-      <c r="G45" s="6" t="n"/>
+      <c r="G46" s="6" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A2:G2"/>
   </mergeCells>
-  <dataValidations count="10">
+  <dataValidations count="11">
     <dataValidation sqref="C13" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"L,C,E"</formula1>
     </dataValidation>
@@ -2416,7 +2445,10 @@
     <dataValidation sqref="C39" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"POISSON,NEGBIN"</formula1>
     </dataValidation>
-    <dataValidation sqref="C45" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="C42" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"LOGNORMAL,NORMAL"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C46" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"QUOTE,USD"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2931,7 +2963,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G49"/>
+  <dimension ref="A1:G64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2953,7 +2985,7 @@
     <row r="2" ht="48" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>CAVEAT: portfolio-level development factors are driven by high-frequency, low-severity claims and may UNDERSTATE development above an attachment point (later reporting, case-estimate movement, slower settlement). Prefer large-claim development or a case review; state the basis. indicated_factor is written by Alteryx (reference only).</t>
+          <t>CAVEAT: portfolio-level development factors are driven by high-frequency, low-severity claims and may UNDERSTATE development above an attachment point (later reporting, case-estimate movement, slower settlement). Prefer large-claim development or a case review; state the basis. ATTRITIONAL: completion of total claims below the stop-loss large threshold (aggregate development, unearned and unwritten), used by the stop-loss attritional model only. indicated_factor is written by Alteryx (reference only).</t>
         </is>
       </c>
     </row>
@@ -3069,12 +3101,12 @@
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>UNEARNED</t>
+          <t>IBNR</t>
         </is>
       </c>
       <c r="C8" s="7" t="inlineStr">
         <is>
-          <t>PRE_AP</t>
+          <t>ATTRITIONAL</t>
         </is>
       </c>
       <c r="D8" s="7" t="n">
@@ -3097,7 +3129,7 @@
       </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
-          <t>POST_AP_AMOUNT</t>
+          <t>PRE_AP</t>
         </is>
       </c>
       <c r="D9" s="7" t="n">
@@ -3120,7 +3152,7 @@
       </c>
       <c r="C10" s="7" t="inlineStr">
         <is>
-          <t>POST_AP_COUNT</t>
+          <t>POST_AP_AMOUNT</t>
         </is>
       </c>
       <c r="D10" s="7" t="n">
@@ -3138,12 +3170,12 @@
       </c>
       <c r="B11" s="7" t="inlineStr">
         <is>
-          <t>UNWRITTEN</t>
+          <t>UNEARNED</t>
         </is>
       </c>
       <c r="C11" s="7" t="inlineStr">
         <is>
-          <t>PRE_AP</t>
+          <t>POST_AP_COUNT</t>
         </is>
       </c>
       <c r="D11" s="7" t="n">
@@ -3161,12 +3193,12 @@
       </c>
       <c r="B12" s="7" t="inlineStr">
         <is>
-          <t>UNWRITTEN</t>
+          <t>UNEARNED</t>
         </is>
       </c>
       <c r="C12" s="7" t="inlineStr">
         <is>
-          <t>POST_AP_AMOUNT</t>
+          <t>ATTRITIONAL</t>
         </is>
       </c>
       <c r="D12" s="7" t="n">
@@ -3189,7 +3221,7 @@
       </c>
       <c r="C13" s="7" t="inlineStr">
         <is>
-          <t>POST_AP_COUNT</t>
+          <t>PRE_AP</t>
         </is>
       </c>
       <c r="D13" s="7" t="n">
@@ -3203,16 +3235,16 @@
     </row>
     <row r="14">
       <c r="A14" s="7" t="n">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="B14" s="7" t="inlineStr">
         <is>
-          <t>IBNR</t>
+          <t>UNWRITTEN</t>
         </is>
       </c>
       <c r="C14" s="7" t="inlineStr">
         <is>
-          <t>PRE_AP</t>
+          <t>POST_AP_AMOUNT</t>
         </is>
       </c>
       <c r="D14" s="7" t="n">
@@ -3226,16 +3258,16 @@
     </row>
     <row r="15">
       <c r="A15" s="7" t="n">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="B15" s="7" t="inlineStr">
         <is>
-          <t>IBNR</t>
+          <t>UNWRITTEN</t>
         </is>
       </c>
       <c r="C15" s="7" t="inlineStr">
         <is>
-          <t>POST_AP_AMOUNT</t>
+          <t>POST_AP_COUNT</t>
         </is>
       </c>
       <c r="D15" s="7" t="n">
@@ -3249,16 +3281,16 @@
     </row>
     <row r="16">
       <c r="A16" s="7" t="n">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="B16" s="7" t="inlineStr">
         <is>
-          <t>IBNR</t>
+          <t>UNWRITTEN</t>
         </is>
       </c>
       <c r="C16" s="7" t="inlineStr">
         <is>
-          <t>POST_AP_COUNT</t>
+          <t>ATTRITIONAL</t>
         </is>
       </c>
       <c r="D16" s="7" t="n">
@@ -3276,7 +3308,7 @@
       </c>
       <c r="B17" s="7" t="inlineStr">
         <is>
-          <t>UNEARNED</t>
+          <t>IBNR</t>
         </is>
       </c>
       <c r="C17" s="7" t="inlineStr">
@@ -3299,7 +3331,7 @@
       </c>
       <c r="B18" s="7" t="inlineStr">
         <is>
-          <t>UNEARNED</t>
+          <t>IBNR</t>
         </is>
       </c>
       <c r="C18" s="7" t="inlineStr">
@@ -3322,7 +3354,7 @@
       </c>
       <c r="B19" s="7" t="inlineStr">
         <is>
-          <t>UNEARNED</t>
+          <t>IBNR</t>
         </is>
       </c>
       <c r="C19" s="7" t="inlineStr">
@@ -3345,12 +3377,12 @@
       </c>
       <c r="B20" s="7" t="inlineStr">
         <is>
-          <t>UNWRITTEN</t>
+          <t>IBNR</t>
         </is>
       </c>
       <c r="C20" s="7" t="inlineStr">
         <is>
-          <t>PRE_AP</t>
+          <t>ATTRITIONAL</t>
         </is>
       </c>
       <c r="D20" s="7" t="n">
@@ -3368,12 +3400,12 @@
       </c>
       <c r="B21" s="7" t="inlineStr">
         <is>
-          <t>UNWRITTEN</t>
+          <t>UNEARNED</t>
         </is>
       </c>
       <c r="C21" s="7" t="inlineStr">
         <is>
-          <t>POST_AP_AMOUNT</t>
+          <t>PRE_AP</t>
         </is>
       </c>
       <c r="D21" s="7" t="n">
@@ -3391,12 +3423,12 @@
       </c>
       <c r="B22" s="7" t="inlineStr">
         <is>
-          <t>UNWRITTEN</t>
+          <t>UNEARNED</t>
         </is>
       </c>
       <c r="C22" s="7" t="inlineStr">
         <is>
-          <t>POST_AP_COUNT</t>
+          <t>POST_AP_AMOUNT</t>
         </is>
       </c>
       <c r="D22" s="7" t="n">
@@ -3410,16 +3442,16 @@
     </row>
     <row r="23">
       <c r="A23" s="7" t="n">
-        <v>2023</v>
+        <v>2022</v>
       </c>
       <c r="B23" s="7" t="inlineStr">
         <is>
-          <t>IBNR</t>
+          <t>UNEARNED</t>
         </is>
       </c>
       <c r="C23" s="7" t="inlineStr">
         <is>
-          <t>PRE_AP</t>
+          <t>POST_AP_COUNT</t>
         </is>
       </c>
       <c r="D23" s="7" t="n">
@@ -3433,16 +3465,16 @@
     </row>
     <row r="24">
       <c r="A24" s="7" t="n">
-        <v>2023</v>
+        <v>2022</v>
       </c>
       <c r="B24" s="7" t="inlineStr">
         <is>
-          <t>IBNR</t>
+          <t>UNEARNED</t>
         </is>
       </c>
       <c r="C24" s="7" t="inlineStr">
         <is>
-          <t>POST_AP_AMOUNT</t>
+          <t>ATTRITIONAL</t>
         </is>
       </c>
       <c r="D24" s="7" t="n">
@@ -3456,16 +3488,16 @@
     </row>
     <row r="25">
       <c r="A25" s="7" t="n">
-        <v>2023</v>
+        <v>2022</v>
       </c>
       <c r="B25" s="7" t="inlineStr">
         <is>
-          <t>IBNR</t>
+          <t>UNWRITTEN</t>
         </is>
       </c>
       <c r="C25" s="7" t="inlineStr">
         <is>
-          <t>POST_AP_COUNT</t>
+          <t>PRE_AP</t>
         </is>
       </c>
       <c r="D25" s="7" t="n">
@@ -3479,16 +3511,16 @@
     </row>
     <row r="26">
       <c r="A26" s="7" t="n">
-        <v>2023</v>
+        <v>2022</v>
       </c>
       <c r="B26" s="7" t="inlineStr">
         <is>
-          <t>UNEARNED</t>
+          <t>UNWRITTEN</t>
         </is>
       </c>
       <c r="C26" s="7" t="inlineStr">
         <is>
-          <t>PRE_AP</t>
+          <t>POST_AP_AMOUNT</t>
         </is>
       </c>
       <c r="D26" s="7" t="n">
@@ -3502,16 +3534,16 @@
     </row>
     <row r="27">
       <c r="A27" s="7" t="n">
-        <v>2023</v>
+        <v>2022</v>
       </c>
       <c r="B27" s="7" t="inlineStr">
         <is>
-          <t>UNEARNED</t>
+          <t>UNWRITTEN</t>
         </is>
       </c>
       <c r="C27" s="7" t="inlineStr">
         <is>
-          <t>POST_AP_AMOUNT</t>
+          <t>POST_AP_COUNT</t>
         </is>
       </c>
       <c r="D27" s="7" t="n">
@@ -3525,16 +3557,16 @@
     </row>
     <row r="28">
       <c r="A28" s="7" t="n">
-        <v>2023</v>
+        <v>2022</v>
       </c>
       <c r="B28" s="7" t="inlineStr">
         <is>
-          <t>UNEARNED</t>
+          <t>UNWRITTEN</t>
         </is>
       </c>
       <c r="C28" s="7" t="inlineStr">
         <is>
-          <t>POST_AP_COUNT</t>
+          <t>ATTRITIONAL</t>
         </is>
       </c>
       <c r="D28" s="7" t="n">
@@ -3552,7 +3584,7 @@
       </c>
       <c r="B29" s="7" t="inlineStr">
         <is>
-          <t>UNWRITTEN</t>
+          <t>IBNR</t>
         </is>
       </c>
       <c r="C29" s="7" t="inlineStr">
@@ -3575,7 +3607,7 @@
       </c>
       <c r="B30" s="7" t="inlineStr">
         <is>
-          <t>UNWRITTEN</t>
+          <t>IBNR</t>
         </is>
       </c>
       <c r="C30" s="7" t="inlineStr">
@@ -3598,7 +3630,7 @@
       </c>
       <c r="B31" s="7" t="inlineStr">
         <is>
-          <t>UNWRITTEN</t>
+          <t>IBNR</t>
         </is>
       </c>
       <c r="C31" s="7" t="inlineStr">
@@ -3617,7 +3649,7 @@
     </row>
     <row r="32">
       <c r="A32" s="7" t="n">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="B32" s="7" t="inlineStr">
         <is>
@@ -3626,7 +3658,7 @@
       </c>
       <c r="C32" s="7" t="inlineStr">
         <is>
-          <t>PRE_AP</t>
+          <t>ATTRITIONAL</t>
         </is>
       </c>
       <c r="D32" s="7" t="n">
@@ -3640,61 +3672,53 @@
     </row>
     <row r="33">
       <c r="A33" s="7" t="n">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="B33" s="7" t="inlineStr">
         <is>
-          <t>IBNR</t>
+          <t>UNEARNED</t>
         </is>
       </c>
       <c r="C33" s="7" t="inlineStr">
         <is>
-          <t>POST_AP_AMOUNT</t>
+          <t>PRE_AP</t>
         </is>
       </c>
       <c r="D33" s="7" t="n">
         <v>0</v>
       </c>
       <c r="E33" s="7" t="n">
-        <v>1.2715</v>
+        <v>1</v>
       </c>
       <c r="F33" s="9" t="n"/>
-      <c r="G33" s="6" t="inlineStr">
-        <is>
-          <t>Synthetic: set from synthetic_truth.json, reference layer 400k xs 100k</t>
-        </is>
-      </c>
+      <c r="G33" s="6" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="7" t="n">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="B34" s="7" t="inlineStr">
         <is>
-          <t>IBNR</t>
+          <t>UNEARNED</t>
         </is>
       </c>
       <c r="C34" s="7" t="inlineStr">
         <is>
-          <t>POST_AP_COUNT</t>
+          <t>POST_AP_AMOUNT</t>
         </is>
       </c>
       <c r="D34" s="7" t="n">
         <v>0</v>
       </c>
       <c r="E34" s="7" t="n">
-        <v>1.1818</v>
+        <v>1</v>
       </c>
       <c r="F34" s="9" t="n"/>
-      <c r="G34" s="6" t="inlineStr">
-        <is>
-          <t>Synthetic: set from synthetic_truth.json, reference layer 400k xs 100k</t>
-        </is>
-      </c>
+      <c r="G34" s="6" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="7" t="n">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="B35" s="7" t="inlineStr">
         <is>
@@ -3703,7 +3727,7 @@
       </c>
       <c r="C35" s="7" t="inlineStr">
         <is>
-          <t>PRE_AP</t>
+          <t>POST_AP_COUNT</t>
         </is>
       </c>
       <c r="D35" s="7" t="n">
@@ -3717,7 +3741,7 @@
     </row>
     <row r="36">
       <c r="A36" s="7" t="n">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="B36" s="7" t="inlineStr">
         <is>
@@ -3726,52 +3750,44 @@
       </c>
       <c r="C36" s="7" t="inlineStr">
         <is>
-          <t>POST_AP_AMOUNT</t>
+          <t>ATTRITIONAL</t>
         </is>
       </c>
       <c r="D36" s="7" t="n">
         <v>0</v>
       </c>
       <c r="E36" s="7" t="n">
-        <v>1.1058</v>
+        <v>1</v>
       </c>
       <c r="F36" s="9" t="n"/>
-      <c r="G36" s="6" t="inlineStr">
-        <is>
-          <t>Synthetic: set from synthetic_truth.json, reference layer 400k xs 100k</t>
-        </is>
-      </c>
+      <c r="G36" s="6" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="7" t="n">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="B37" s="7" t="inlineStr">
         <is>
-          <t>UNEARNED</t>
+          <t>UNWRITTEN</t>
         </is>
       </c>
       <c r="C37" s="7" t="inlineStr">
         <is>
-          <t>POST_AP_COUNT</t>
+          <t>PRE_AP</t>
         </is>
       </c>
       <c r="D37" s="7" t="n">
         <v>0</v>
       </c>
       <c r="E37" s="7" t="n">
-        <v>1.0256</v>
+        <v>1</v>
       </c>
       <c r="F37" s="9" t="n"/>
-      <c r="G37" s="6" t="inlineStr">
-        <is>
-          <t>Synthetic: set from synthetic_truth.json, reference layer 400k xs 100k</t>
-        </is>
-      </c>
+      <c r="G37" s="6" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="7" t="n">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="B38" s="7" t="inlineStr">
         <is>
@@ -3780,7 +3796,7 @@
       </c>
       <c r="C38" s="7" t="inlineStr">
         <is>
-          <t>PRE_AP</t>
+          <t>POST_AP_AMOUNT</t>
         </is>
       </c>
       <c r="D38" s="7" t="n">
@@ -3794,7 +3810,7 @@
     </row>
     <row r="39">
       <c r="A39" s="7" t="n">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="B39" s="7" t="inlineStr">
         <is>
@@ -3803,7 +3819,7 @@
       </c>
       <c r="C39" s="7" t="inlineStr">
         <is>
-          <t>POST_AP_AMOUNT</t>
+          <t>POST_AP_COUNT</t>
         </is>
       </c>
       <c r="D39" s="7" t="n">
@@ -3817,7 +3833,7 @@
     </row>
     <row r="40">
       <c r="A40" s="7" t="n">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="B40" s="7" t="inlineStr">
         <is>
@@ -3826,7 +3842,7 @@
       </c>
       <c r="C40" s="7" t="inlineStr">
         <is>
-          <t>POST_AP_COUNT</t>
+          <t>ATTRITIONAL</t>
         </is>
       </c>
       <c r="D40" s="7" t="n">
@@ -3840,7 +3856,7 @@
     </row>
     <row r="41">
       <c r="A41" s="7" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="B41" s="7" t="inlineStr">
         <is>
@@ -3863,7 +3879,7 @@
     </row>
     <row r="42">
       <c r="A42" s="7" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="B42" s="7" t="inlineStr">
         <is>
@@ -3879,7 +3895,7 @@
         <v>0</v>
       </c>
       <c r="E42" s="7" t="n">
-        <v>2.687</v>
+        <v>1.2715</v>
       </c>
       <c r="F42" s="9" t="n"/>
       <c r="G42" s="6" t="inlineStr">
@@ -3890,7 +3906,7 @@
     </row>
     <row r="43">
       <c r="A43" s="7" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="B43" s="7" t="inlineStr">
         <is>
@@ -3906,7 +3922,7 @@
         <v>0</v>
       </c>
       <c r="E43" s="7" t="n">
-        <v>1.5833</v>
+        <v>1.1818</v>
       </c>
       <c r="F43" s="9" t="n"/>
       <c r="G43" s="6" t="inlineStr">
@@ -3917,30 +3933,34 @@
     </row>
     <row r="44">
       <c r="A44" s="7" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="B44" s="7" t="inlineStr">
         <is>
-          <t>UNEARNED</t>
+          <t>IBNR</t>
         </is>
       </c>
       <c r="C44" s="7" t="inlineStr">
         <is>
-          <t>PRE_AP</t>
+          <t>ATTRITIONAL</t>
         </is>
       </c>
       <c r="D44" s="7" t="n">
         <v>0</v>
       </c>
       <c r="E44" s="7" t="n">
-        <v>1</v>
+        <v>1.0754</v>
       </c>
       <c r="F44" s="9" t="n"/>
-      <c r="G44" s="6" t="n"/>
+      <c r="G44" s="6" t="inlineStr">
+        <is>
+          <t>Synthetic: set from synthetic_truth.json, total claims</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="7" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="B45" s="7" t="inlineStr">
         <is>
@@ -3949,25 +3969,21 @@
       </c>
       <c r="C45" s="7" t="inlineStr">
         <is>
-          <t>POST_AP_AMOUNT</t>
+          <t>PRE_AP</t>
         </is>
       </c>
       <c r="D45" s="7" t="n">
         <v>0</v>
       </c>
       <c r="E45" s="7" t="n">
-        <v>1.9676</v>
+        <v>1</v>
       </c>
       <c r="F45" s="9" t="n"/>
-      <c r="G45" s="6" t="inlineStr">
-        <is>
-          <t>Synthetic: set from synthetic_truth.json, reference layer 400k xs 100k</t>
-        </is>
-      </c>
+      <c r="G45" s="6" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="7" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="B46" s="7" t="inlineStr">
         <is>
@@ -3976,14 +3992,14 @@
       </c>
       <c r="C46" s="7" t="inlineStr">
         <is>
-          <t>POST_AP_COUNT</t>
+          <t>POST_AP_AMOUNT</t>
         </is>
       </c>
       <c r="D46" s="7" t="n">
         <v>0</v>
       </c>
       <c r="E46" s="7" t="n">
-        <v>2.5263</v>
+        <v>1.1058</v>
       </c>
       <c r="F46" s="9" t="n"/>
       <c r="G46" s="6" t="inlineStr">
@@ -3994,78 +4010,459 @@
     </row>
     <row r="47">
       <c r="A47" s="7" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="B47" s="7" t="inlineStr">
         <is>
-          <t>UNWRITTEN</t>
+          <t>UNEARNED</t>
         </is>
       </c>
       <c r="C47" s="7" t="inlineStr">
         <is>
-          <t>PRE_AP</t>
+          <t>POST_AP_COUNT</t>
         </is>
       </c>
       <c r="D47" s="7" t="n">
         <v>0</v>
       </c>
       <c r="E47" s="7" t="n">
-        <v>1</v>
+        <v>1.0256</v>
       </c>
       <c r="F47" s="9" t="n"/>
-      <c r="G47" s="6" t="n"/>
+      <c r="G47" s="6" t="inlineStr">
+        <is>
+          <t>Synthetic: set from synthetic_truth.json, reference layer 400k xs 100k</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="7" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="B48" s="7" t="inlineStr">
         <is>
-          <t>UNWRITTEN</t>
+          <t>UNEARNED</t>
         </is>
       </c>
       <c r="C48" s="7" t="inlineStr">
         <is>
-          <t>POST_AP_AMOUNT</t>
+          <t>ATTRITIONAL</t>
         </is>
       </c>
       <c r="D48" s="7" t="n">
         <v>0</v>
       </c>
       <c r="E48" s="7" t="n">
-        <v>1.1908</v>
+        <v>1.0368</v>
       </c>
       <c r="F48" s="9" t="n"/>
       <c r="G48" s="6" t="inlineStr">
         <is>
-          <t>Synthetic: set from synthetic_truth.json, reference layer 400k xs 100k</t>
+          <t>Synthetic: set from synthetic_truth.json, total claims</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="7" t="n">
+        <v>2024</v>
+      </c>
+      <c r="B49" s="7" t="inlineStr">
+        <is>
+          <t>UNWRITTEN</t>
+        </is>
+      </c>
+      <c r="C49" s="7" t="inlineStr">
+        <is>
+          <t>PRE_AP</t>
+        </is>
+      </c>
+      <c r="D49" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E49" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F49" s="9" t="n"/>
+      <c r="G49" s="6" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="7" t="n">
+        <v>2024</v>
+      </c>
+      <c r="B50" s="7" t="inlineStr">
+        <is>
+          <t>UNWRITTEN</t>
+        </is>
+      </c>
+      <c r="C50" s="7" t="inlineStr">
+        <is>
+          <t>POST_AP_AMOUNT</t>
+        </is>
+      </c>
+      <c r="D50" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E50" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F50" s="9" t="n"/>
+      <c r="G50" s="6" t="n"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="7" t="n">
+        <v>2024</v>
+      </c>
+      <c r="B51" s="7" t="inlineStr">
+        <is>
+          <t>UNWRITTEN</t>
+        </is>
+      </c>
+      <c r="C51" s="7" t="inlineStr">
+        <is>
+          <t>POST_AP_COUNT</t>
+        </is>
+      </c>
+      <c r="D51" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E51" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F51" s="9" t="n"/>
+      <c r="G51" s="6" t="n"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="7" t="n">
+        <v>2024</v>
+      </c>
+      <c r="B52" s="7" t="inlineStr">
+        <is>
+          <t>UNWRITTEN</t>
+        </is>
+      </c>
+      <c r="C52" s="7" t="inlineStr">
+        <is>
+          <t>ATTRITIONAL</t>
+        </is>
+      </c>
+      <c r="D52" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E52" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F52" s="9" t="n"/>
+      <c r="G52" s="6" t="n"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="7" t="n">
         <v>2025</v>
       </c>
-      <c r="B49" s="7" t="inlineStr">
+      <c r="B53" s="7" t="inlineStr">
+        <is>
+          <t>IBNR</t>
+        </is>
+      </c>
+      <c r="C53" s="7" t="inlineStr">
+        <is>
+          <t>PRE_AP</t>
+        </is>
+      </c>
+      <c r="D53" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E53" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F53" s="9" t="n"/>
+      <c r="G53" s="6" t="n"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="7" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B54" s="7" t="inlineStr">
+        <is>
+          <t>IBNR</t>
+        </is>
+      </c>
+      <c r="C54" s="7" t="inlineStr">
+        <is>
+          <t>POST_AP_AMOUNT</t>
+        </is>
+      </c>
+      <c r="D54" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E54" s="7" t="n">
+        <v>2.687</v>
+      </c>
+      <c r="F54" s="9" t="n"/>
+      <c r="G54" s="6" t="inlineStr">
+        <is>
+          <t>Synthetic: set from synthetic_truth.json, reference layer 400k xs 100k</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="7" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B55" s="7" t="inlineStr">
+        <is>
+          <t>IBNR</t>
+        </is>
+      </c>
+      <c r="C55" s="7" t="inlineStr">
+        <is>
+          <t>POST_AP_COUNT</t>
+        </is>
+      </c>
+      <c r="D55" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E55" s="7" t="n">
+        <v>1.5833</v>
+      </c>
+      <c r="F55" s="9" t="n"/>
+      <c r="G55" s="6" t="inlineStr">
+        <is>
+          <t>Synthetic: set from synthetic_truth.json, reference layer 400k xs 100k</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="7" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B56" s="7" t="inlineStr">
+        <is>
+          <t>IBNR</t>
+        </is>
+      </c>
+      <c r="C56" s="7" t="inlineStr">
+        <is>
+          <t>ATTRITIONAL</t>
+        </is>
+      </c>
+      <c r="D56" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E56" s="7" t="n">
+        <v>1.4774</v>
+      </c>
+      <c r="F56" s="9" t="n"/>
+      <c r="G56" s="6" t="inlineStr">
+        <is>
+          <t>Synthetic: set from synthetic_truth.json, total claims</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="7" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B57" s="7" t="inlineStr">
+        <is>
+          <t>UNEARNED</t>
+        </is>
+      </c>
+      <c r="C57" s="7" t="inlineStr">
+        <is>
+          <t>PRE_AP</t>
+        </is>
+      </c>
+      <c r="D57" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E57" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F57" s="9" t="n"/>
+      <c r="G57" s="6" t="n"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="7" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B58" s="7" t="inlineStr">
+        <is>
+          <t>UNEARNED</t>
+        </is>
+      </c>
+      <c r="C58" s="7" t="inlineStr">
+        <is>
+          <t>POST_AP_AMOUNT</t>
+        </is>
+      </c>
+      <c r="D58" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E58" s="7" t="n">
+        <v>1.9676</v>
+      </c>
+      <c r="F58" s="9" t="n"/>
+      <c r="G58" s="6" t="inlineStr">
+        <is>
+          <t>Synthetic: set from synthetic_truth.json, reference layer 400k xs 100k</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="7" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B59" s="7" t="inlineStr">
+        <is>
+          <t>UNEARNED</t>
+        </is>
+      </c>
+      <c r="C59" s="7" t="inlineStr">
+        <is>
+          <t>POST_AP_COUNT</t>
+        </is>
+      </c>
+      <c r="D59" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E59" s="7" t="n">
+        <v>2.5263</v>
+      </c>
+      <c r="F59" s="9" t="n"/>
+      <c r="G59" s="6" t="inlineStr">
+        <is>
+          <t>Synthetic: set from synthetic_truth.json, reference layer 400k xs 100k</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="7" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B60" s="7" t="inlineStr">
+        <is>
+          <t>UNEARNED</t>
+        </is>
+      </c>
+      <c r="C60" s="7" t="inlineStr">
+        <is>
+          <t>ATTRITIONAL</t>
+        </is>
+      </c>
+      <c r="D60" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E60" s="7" t="n">
+        <v>2.2749</v>
+      </c>
+      <c r="F60" s="9" t="n"/>
+      <c r="G60" s="6" t="inlineStr">
+        <is>
+          <t>Synthetic: set from synthetic_truth.json, total claims</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="7" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B61" s="7" t="inlineStr">
         <is>
           <t>UNWRITTEN</t>
         </is>
       </c>
-      <c r="C49" s="7" t="inlineStr">
+      <c r="C61" s="7" t="inlineStr">
+        <is>
+          <t>PRE_AP</t>
+        </is>
+      </c>
+      <c r="D61" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E61" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F61" s="9" t="n"/>
+      <c r="G61" s="6" t="n"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="7" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B62" s="7" t="inlineStr">
+        <is>
+          <t>UNWRITTEN</t>
+        </is>
+      </c>
+      <c r="C62" s="7" t="inlineStr">
+        <is>
+          <t>POST_AP_AMOUNT</t>
+        </is>
+      </c>
+      <c r="D62" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E62" s="7" t="n">
+        <v>1.1908</v>
+      </c>
+      <c r="F62" s="9" t="n"/>
+      <c r="G62" s="6" t="inlineStr">
+        <is>
+          <t>Synthetic: set from synthetic_truth.json, reference layer 400k xs 100k</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="7" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B63" s="7" t="inlineStr">
+        <is>
+          <t>UNWRITTEN</t>
+        </is>
+      </c>
+      <c r="C63" s="7" t="inlineStr">
         <is>
           <t>POST_AP_COUNT</t>
         </is>
       </c>
-      <c r="D49" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="E49" s="7" t="n">
+      <c r="D63" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E63" s="7" t="n">
         <v>1.25</v>
       </c>
-      <c r="F49" s="9" t="n"/>
-      <c r="G49" s="6" t="inlineStr">
+      <c r="F63" s="9" t="n"/>
+      <c r="G63" s="6" t="inlineStr">
         <is>
           <t>Synthetic: set from synthetic_truth.json, reference layer 400k xs 100k</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="7" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B64" s="7" t="inlineStr">
+        <is>
+          <t>UNWRITTEN</t>
+        </is>
+      </c>
+      <c r="C64" s="7" t="inlineStr">
+        <is>
+          <t>ATTRITIONAL</t>
+        </is>
+      </c>
+      <c r="D64" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E64" s="7" t="n">
+        <v>1.3165</v>
+      </c>
+      <c r="F64" s="9" t="n"/>
+      <c r="G64" s="6" t="inlineStr">
+        <is>
+          <t>Synthetic: set from synthetic_truth.json, total claims</t>
         </is>
       </c>
     </row>
@@ -4074,11 +4471,11 @@
     <mergeCell ref="A2:G2"/>
   </mergeCells>
   <dataValidations count="2">
-    <dataValidation sqref="B5:B54" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="B5:B64" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"IBNR,UNEARNED,UNWRITTEN"</formula1>
     </dataValidation>
-    <dataValidation sqref="C5:C54" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"PRE_AP,POST_AP_AMOUNT,POST_AP_COUNT"</formula1>
+    <dataValidation sqref="C5:C64" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"PRE_AP,POST_AP_AMOUNT,POST_AP_COUNT,ATTRITIONAL"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
WIP 0.5: stage 04a severity fit (Python tool), engine runner
- tools/python/sevfit.py: left-truncated, right-censored MLE of LOGNORMAL, GAMMA, WEIBULL,
  PARETO, GPD; AIC/BIC, KS vs Kaplan-Meier, mean excess at APs, boundary-fit flag,
  selection (fit_selected, else lowest AIC), inverse-survival grid.
- 04a_fit_severity.yxmd (Python tool, XML as Designer 2026.2 saves it); stage 04 draws
  severity from the grid (severity_source PYTHON/NATIVE; native Pareto exact on the grid);
  stage 03 resets the fit; check S07; params fit_selected, severity_source.
- Simulator: Python tool emulation, Log10. Results workbook: Severity sheet and fit data sheets.
- tests/test_sevfit.py; stage 04/06/07 tests extended (simulator: pass).
- tools/run_pipeline.bat: runs all workflows with AlteryxEngineCmd.exe.
Pending: Designer/engine run of 04a-07, twin re-baseline, docs.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UTL5cPxKguFWxKSpgQZCbz
</commit_message>
<xml_diff>
--- a/data/synthetic/XoL_Control_synthetic.xlsx
+++ b/data/synthetic/XoL_Control_synthetic.xlsx
@@ -1204,7 +1204,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G48"/>
+  <dimension ref="A1:G50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2221,7 +2221,7 @@
     <row r="40">
       <c r="A40" s="5" t="inlineStr">
         <is>
-          <t>freq_model</t>
+          <t>fit_selected</t>
         </is>
       </c>
       <c r="B40" s="5" t="inlineStr">
@@ -2229,20 +2229,16 @@
           <t>Stochastic</t>
         </is>
       </c>
-      <c r="C40" s="6" t="inlineStr">
-        <is>
-          <t>POISSON</t>
-        </is>
-      </c>
+      <c r="C40" s="6" t="n"/>
       <c r="D40" s="5" t="inlineStr"/>
       <c r="E40" s="5" t="inlineStr">
         <is>
-          <t>POISSON,NEGBIN</t>
+          <t>LOGNORMAL,GAMMA,WEIBULL,PARETO,GPD</t>
         </is>
       </c>
       <c r="F40" s="5" t="inlineStr">
         <is>
-          <t>Frequency distribution [required]</t>
+          <t>Severity distribution used by the simulation (blank = lowest AIC in stage 04a); justify an override</t>
         </is>
       </c>
       <c r="G40" s="6" t="n"/>
@@ -2250,7 +2246,7 @@
     <row r="41">
       <c r="A41" s="5" t="inlineStr">
         <is>
-          <t>ev_freq_source</t>
+          <t>severity_source</t>
         </is>
       </c>
       <c r="B41" s="5" t="inlineStr">
@@ -2260,18 +2256,18 @@
       </c>
       <c r="C41" s="6" t="inlineStr">
         <is>
-          <t>BOTH</t>
+          <t>PYTHON</t>
         </is>
       </c>
       <c r="D41" s="5" t="inlineStr"/>
       <c r="E41" s="5" t="inlineStr">
         <is>
-          <t>EXPERIENCE,SCENARIOS,BOTH</t>
+          <t>PYTHON,NATIVE</t>
         </is>
       </c>
       <c r="F41" s="5" t="inlineStr">
         <is>
-          <t>Per-event simulation: historical events, EvScenarios (with a return period), or both [required]</t>
+          <t>PYTHON: distribution selected in 04a_fit_severity (Python tool); NATIVE: Pareto fitted in stage 04 (no Python) [required]</t>
         </is>
       </c>
       <c r="G41" s="6" t="n"/>
@@ -2279,7 +2275,7 @@
     <row r="42">
       <c r="A42" s="5" t="inlineStr">
         <is>
-          <t>sl_attritional_threshold</t>
+          <t>freq_model</t>
         </is>
       </c>
       <c r="B42" s="5" t="inlineStr">
@@ -2289,18 +2285,18 @@
       </c>
       <c r="C42" s="6" t="inlineStr">
         <is>
-          <t>100000</t>
-        </is>
-      </c>
-      <c r="D42" s="5" t="inlineStr">
-        <is>
-          <t>quote ccy</t>
-        </is>
-      </c>
-      <c r="E42" s="5" t="inlineStr"/>
+          <t>POISSON</t>
+        </is>
+      </c>
+      <c r="D42" s="5" t="inlineStr"/>
+      <c r="E42" s="5" t="inlineStr">
+        <is>
+          <t>POISSON,NEGBIN</t>
+        </is>
+      </c>
       <c r="F42" s="5" t="inlineStr">
         <is>
-          <t>Stop loss: attritional / large split [required]</t>
+          <t>Frequency distribution [required]</t>
         </is>
       </c>
       <c r="G42" s="6" t="n"/>
@@ -2308,7 +2304,7 @@
     <row r="43">
       <c r="A43" s="5" t="inlineStr">
         <is>
-          <t>sl_cov_floor</t>
+          <t>ev_freq_source</t>
         </is>
       </c>
       <c r="B43" s="5" t="inlineStr">
@@ -2318,14 +2314,18 @@
       </c>
       <c r="C43" s="6" t="inlineStr">
         <is>
-          <t>0.05</t>
+          <t>BOTH</t>
         </is>
       </c>
       <c r="D43" s="5" t="inlineStr"/>
-      <c r="E43" s="5" t="inlineStr"/>
+      <c r="E43" s="5" t="inlineStr">
+        <is>
+          <t>EXPERIENCE,SCENARIOS,BOTH</t>
+        </is>
+      </c>
       <c r="F43" s="5" t="inlineStr">
         <is>
-          <t>Stop loss: minimum CoV of the attritional cost per life [required]</t>
+          <t>Per-event simulation: historical events, EvScenarios (with a return period), or both [required]</t>
         </is>
       </c>
       <c r="G43" s="6" t="n"/>
@@ -2333,7 +2333,7 @@
     <row r="44">
       <c r="A44" s="5" t="inlineStr">
         <is>
-          <t>sl_attritional_dist</t>
+          <t>sl_attritional_threshold</t>
         </is>
       </c>
       <c r="B44" s="5" t="inlineStr">
@@ -2343,18 +2343,18 @@
       </c>
       <c r="C44" s="6" t="inlineStr">
         <is>
-          <t>LOGNORMAL</t>
-        </is>
-      </c>
-      <c r="D44" s="5" t="inlineStr"/>
-      <c r="E44" s="5" t="inlineStr">
-        <is>
-          <t>LOGNORMAL,NORMAL</t>
-        </is>
-      </c>
+          <t>100000</t>
+        </is>
+      </c>
+      <c r="D44" s="5" t="inlineStr">
+        <is>
+          <t>quote ccy</t>
+        </is>
+      </c>
+      <c r="E44" s="5" t="inlineStr"/>
       <c r="F44" s="5" t="inlineStr">
         <is>
-          <t>Stop loss: distribution of the attritional cost per life [required]</t>
+          <t>Stop loss: attritional / large split [required]</t>
         </is>
       </c>
       <c r="G44" s="6" t="n"/>
@@ -2362,24 +2362,24 @@
     <row r="45">
       <c r="A45" s="5" t="inlineStr">
         <is>
-          <t>net_claims_budget</t>
+          <t>sl_cov_floor</t>
         </is>
       </c>
       <c r="B45" s="5" t="inlineStr">
         <is>
-          <t>Cedant impact</t>
-        </is>
-      </c>
-      <c r="C45" s="6" t="n"/>
-      <c r="D45" s="5" t="inlineStr">
-        <is>
-          <t>quote ccy</t>
-        </is>
-      </c>
+          <t>Stochastic</t>
+        </is>
+      </c>
+      <c r="C45" s="6" t="inlineStr">
+        <is>
+          <t>0.05</t>
+        </is>
+      </c>
+      <c r="D45" s="5" t="inlineStr"/>
       <c r="E45" s="5" t="inlineStr"/>
       <c r="F45" s="5" t="inlineStr">
         <is>
-          <t>Blank = best-estimate gross claims</t>
+          <t>Stop loss: minimum CoV of the attritional cost per life [required]</t>
         </is>
       </c>
       <c r="G45" s="6" t="n"/>
@@ -2387,24 +2387,28 @@
     <row r="46">
       <c r="A46" s="5" t="inlineStr">
         <is>
-          <t>reference_lives</t>
+          <t>sl_attritional_dist</t>
         </is>
       </c>
       <c r="B46" s="5" t="inlineStr">
         <is>
-          <t>Cedant impact</t>
-        </is>
-      </c>
-      <c r="C46" s="6" t="inlineStr"/>
-      <c r="D46" s="5" t="inlineStr">
-        <is>
-          <t>lives</t>
-        </is>
-      </c>
-      <c r="E46" s="5" t="inlineStr"/>
+          <t>Stochastic</t>
+        </is>
+      </c>
+      <c r="C46" s="6" t="inlineStr">
+        <is>
+          <t>LOGNORMAL</t>
+        </is>
+      </c>
+      <c r="D46" s="5" t="inlineStr"/>
+      <c r="E46" s="5" t="inlineStr">
+        <is>
+          <t>LOGNORMAL,NORMAL</t>
+        </is>
+      </c>
       <c r="F46" s="5" t="inlineStr">
         <is>
-          <t>Blank = expected lives for the quote year</t>
+          <t>Stop loss: distribution of the attritional cost per life [required]</t>
         </is>
       </c>
       <c r="G46" s="6" t="n"/>
@@ -2412,7 +2416,7 @@
     <row r="47">
       <c r="A47" s="5" t="inlineStr">
         <is>
-          <t>return_periods</t>
+          <t>net_claims_budget</t>
         </is>
       </c>
       <c r="B47" s="5" t="inlineStr">
@@ -2420,20 +2424,16 @@
           <t>Cedant impact</t>
         </is>
       </c>
-      <c r="C47" s="6" t="inlineStr">
-        <is>
-          <t>5,50,250</t>
-        </is>
-      </c>
+      <c r="C47" s="6" t="n"/>
       <c r="D47" s="5" t="inlineStr">
         <is>
-          <t>years</t>
+          <t>quote ccy</t>
         </is>
       </c>
       <c r="E47" s="5" t="inlineStr"/>
       <c r="F47" s="5" t="inlineStr">
         <is>
-          <t>Return periods shown in Exhibit C2 [required]</t>
+          <t>Blank = best-estimate gross claims</t>
         </is>
       </c>
       <c r="G47" s="6" t="n"/>
@@ -2441,37 +2441,91 @@
     <row r="48">
       <c r="A48" s="5" t="inlineStr">
         <is>
+          <t>reference_lives</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="inlineStr">
+        <is>
+          <t>Cedant impact</t>
+        </is>
+      </c>
+      <c r="C48" s="6" t="inlineStr"/>
+      <c r="D48" s="5" t="inlineStr">
+        <is>
+          <t>lives</t>
+        </is>
+      </c>
+      <c r="E48" s="5" t="inlineStr"/>
+      <c r="F48" s="5" t="inlineStr">
+        <is>
+          <t>Blank = expected lives for the quote year</t>
+        </is>
+      </c>
+      <c r="G48" s="6" t="n"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>return_periods</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="inlineStr">
+        <is>
+          <t>Cedant impact</t>
+        </is>
+      </c>
+      <c r="C49" s="6" t="inlineStr">
+        <is>
+          <t>5,50,250</t>
+        </is>
+      </c>
+      <c r="D49" s="5" t="inlineStr">
+        <is>
+          <t>years</t>
+        </is>
+      </c>
+      <c r="E49" s="5" t="inlineStr"/>
+      <c r="F49" s="5" t="inlineStr">
+        <is>
+          <t>Return periods shown in Exhibit C2 [required]</t>
+        </is>
+      </c>
+      <c r="G49" s="6" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
           <t>currency_display</t>
         </is>
       </c>
-      <c r="B48" s="5" t="inlineStr">
+      <c r="B50" s="5" t="inlineStr">
         <is>
           <t>Cedant impact</t>
         </is>
       </c>
-      <c r="C48" s="6" t="inlineStr">
+      <c r="C50" s="6" t="inlineStr">
         <is>
           <t>QUOTE</t>
         </is>
       </c>
-      <c r="D48" s="5" t="inlineStr"/>
-      <c r="E48" s="5" t="inlineStr">
+      <c r="D50" s="5" t="inlineStr"/>
+      <c r="E50" s="5" t="inlineStr">
         <is>
           <t>QUOTE,USD</t>
         </is>
       </c>
-      <c r="F48" s="5" t="inlineStr">
+      <c r="F50" s="5" t="inlineStr">
         <is>
           <t>Currency of the client exhibits [required]</t>
         </is>
       </c>
-      <c r="G48" s="6" t="n"/>
+      <c r="G50" s="6" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A2:G2"/>
   </mergeCells>
-  <dataValidations count="12">
+  <dataValidations count="14">
     <dataValidation sqref="C14" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"L,C,E"</formula1>
     </dataValidation>
@@ -2497,15 +2551,21 @@
       <formula1>"STANDALONE,PROGRAMME"</formula1>
     </dataValidation>
     <dataValidation sqref="C40" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"LOGNORMAL,GAMMA,WEIBULL,PARETO,GPD"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C41" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"PYTHON,NATIVE"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C42" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"POISSON,NEGBIN"</formula1>
     </dataValidation>
-    <dataValidation sqref="C41" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="C43" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"EXPERIENCE,SCENARIOS,BOTH"</formula1>
     </dataValidation>
-    <dataValidation sqref="C44" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="C46" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"LOGNORMAL,NORMAL"</formula1>
     </dataValidation>
-    <dataValidation sqref="C48" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="C50" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"QUOTE,USD"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
WIP 0.6: Merit v7 final outputs as an input (adapter 01c)
- 01c reads Merit's dim_life / fact_member_month / fact_claims / run_manifest_claims as written:
  life-period grain (LifeKey x UWY), valuation date from the manifest, claims after it
  excluded (A04 FLAG), ete_payer_filter + A16, void life-periods kept without exposure (A17).
- tools/import_merit.bat, tools/check_merit.bat, run_pipeline.bat last-stage argument.
- tests/test_merit.py + fixture tests/fixtures/merit_v7 (Merit v7.0.2 synthetic outputs, names
  scrubbed by tools/synth/merit_fixture.py): all checks pass in the simulator.
Pending: engine run on the laptop (check_merit.bat), 01c twin re-baseline, full suite.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UTL5cPxKguFWxKSpgQZCbz
</commit_message>
<xml_diff>
--- a/data/synthetic/XoL_Control_synthetic.xlsx
+++ b/data/synthetic/XoL_Control_synthetic.xlsx
@@ -1204,7 +1204,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G50"/>
+  <dimension ref="A1:G51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1611,28 +1611,20 @@
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>treaty_basis</t>
+          <t>ete_payer_filter</t>
         </is>
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>Basis</t>
-        </is>
-      </c>
-      <c r="C18" s="6" t="inlineStr">
-        <is>
-          <t>RA</t>
-        </is>
-      </c>
+          <t>Mode</t>
+        </is>
+      </c>
+      <c r="C18" s="6" t="n"/>
       <c r="D18" s="5" t="inlineStr"/>
-      <c r="E18" s="5" t="inlineStr">
-        <is>
-          <t>RA,LO</t>
-        </is>
-      </c>
+      <c r="E18" s="5" t="inlineStr"/>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>Risks attaching or losses occurring [required]</t>
+          <t>ETE / Merit only: comma list of payers (Payer Name) to include (blank = all; A16 flags several payers)</t>
         </is>
       </c>
       <c r="G18" s="6" t="n"/>
@@ -1640,7 +1632,7 @@
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>claims_trigger</t>
+          <t>treaty_basis</t>
         </is>
       </c>
       <c r="B19" s="5" t="inlineStr">
@@ -1650,18 +1642,18 @@
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>INCURRED</t>
+          <t>RA</t>
         </is>
       </c>
       <c r="D19" s="5" t="inlineStr"/>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t>INCURRED,PAID</t>
+          <t>RA,LO</t>
         </is>
       </c>
       <c r="F19" s="5" t="inlineStr">
         <is>
-          <t>Claims date trigger [required]</t>
+          <t>Risks attaching or losses occurring [required]</t>
         </is>
       </c>
       <c r="G19" s="6" t="n"/>
@@ -1669,7 +1661,7 @@
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t>paid_runoff_months</t>
+          <t>claims_trigger</t>
         </is>
       </c>
       <c r="B20" s="5" t="inlineStr">
@@ -1677,16 +1669,20 @@
           <t>Basis</t>
         </is>
       </c>
-      <c r="C20" s="6" t="n"/>
-      <c r="D20" s="5" t="inlineStr">
-        <is>
-          <t>months</t>
-        </is>
-      </c>
-      <c r="E20" s="5" t="inlineStr"/>
+      <c r="C20" s="6" t="inlineStr">
+        <is>
+          <t>INCURRED</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="inlineStr"/>
+      <c r="E20" s="5" t="inlineStr">
+        <is>
+          <t>INCURRED,PAID</t>
+        </is>
+      </c>
       <c r="F20" s="5" t="inlineStr">
         <is>
-          <t>Paid trigger only: months after treaty year end</t>
+          <t>Claims date trigger [required]</t>
         </is>
       </c>
       <c r="G20" s="6" t="n"/>
@@ -1694,7 +1690,7 @@
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
-          <t>pp_accumulation</t>
+          <t>paid_runoff_months</t>
         </is>
       </c>
       <c r="B21" s="5" t="inlineStr">
@@ -1702,20 +1698,16 @@
           <t>Basis</t>
         </is>
       </c>
-      <c r="C21" s="6" t="inlineStr">
-        <is>
-          <t>POLICY_YEAR</t>
-        </is>
-      </c>
-      <c r="D21" s="5" t="inlineStr"/>
-      <c r="E21" s="5" t="inlineStr">
-        <is>
-          <t>POLICY_YEAR,TREATY_YEAR</t>
-        </is>
-      </c>
+      <c r="C21" s="6" t="n"/>
+      <c r="D21" s="5" t="inlineStr">
+        <is>
+          <t>months</t>
+        </is>
+      </c>
+      <c r="E21" s="5" t="inlineStr"/>
       <c r="F21" s="5" t="inlineStr">
         <is>
-          <t>Per-person accumulation period [required]</t>
+          <t>Paid trigger only: months after treaty year end</t>
         </is>
       </c>
       <c r="G21" s="6" t="n"/>
@@ -1723,28 +1715,28 @@
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>epi_quote_year</t>
+          <t>pp_accumulation</t>
         </is>
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>Exposure</t>
+          <t>Basis</t>
         </is>
       </c>
       <c r="C22" s="6" t="inlineStr">
         <is>
-          <t>65282847</t>
-        </is>
-      </c>
-      <c r="D22" s="5" t="inlineStr">
-        <is>
-          <t>quote ccy</t>
-        </is>
-      </c>
-      <c r="E22" s="5" t="inlineStr"/>
+          <t>POLICY_YEAR</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="inlineStr"/>
+      <c r="E22" s="5" t="inlineStr">
+        <is>
+          <t>POLICY_YEAR,TREATY_YEAR</t>
+        </is>
+      </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>Expected premium income for the quote year [required]</t>
+          <t>Per-person accumulation period [required]</t>
         </is>
       </c>
       <c r="G22" s="6" t="n"/>
@@ -1752,7 +1744,7 @@
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
         <is>
-          <t>expected_lives_quote_year</t>
+          <t>epi_quote_year</t>
         </is>
       </c>
       <c r="B23" s="5" t="inlineStr">
@@ -1760,16 +1752,20 @@
           <t>Exposure</t>
         </is>
       </c>
-      <c r="C23" s="6" t="n"/>
+      <c r="C23" s="6" t="inlineStr">
+        <is>
+          <t>65282847</t>
+        </is>
+      </c>
       <c r="D23" s="5" t="inlineStr">
         <is>
-          <t>lives</t>
+          <t>quote ccy</t>
         </is>
       </c>
       <c r="E23" s="5" t="inlineStr"/>
       <c r="F23" s="5" t="inlineStr">
         <is>
-          <t>Blank = EPI / trended average premium</t>
+          <t>Expected premium income for the quote year [required]</t>
         </is>
       </c>
       <c r="G23" s="6" t="n"/>
@@ -1777,28 +1773,24 @@
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>years_included</t>
+          <t>expected_lives_quote_year</t>
         </is>
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>Data</t>
-        </is>
-      </c>
-      <c r="C24" s="6" t="inlineStr">
-        <is>
-          <t>2021,2022,2023,2024,2025</t>
-        </is>
-      </c>
+          <t>Exposure</t>
+        </is>
+      </c>
+      <c r="C24" s="6" t="n"/>
       <c r="D24" s="5" t="inlineStr">
         <is>
-          <t>years</t>
+          <t>lives</t>
         </is>
       </c>
       <c r="E24" s="5" t="inlineStr"/>
       <c r="F24" s="5" t="inlineStr">
         <is>
-          <t>Experience years used (comma list, 2-5 years) [required]</t>
+          <t>Blank = EPI / trended average premium</t>
         </is>
       </c>
       <c r="G24" s="6" t="n"/>
@@ -1806,7 +1798,7 @@
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
         <is>
-          <t>output_threshold_pct_min_ap</t>
+          <t>years_included</t>
         </is>
       </c>
       <c r="B25" s="5" t="inlineStr">
@@ -1816,18 +1808,18 @@
       </c>
       <c r="C25" s="6" t="inlineStr">
         <is>
-          <t>0.5</t>
+          <t>2021,2022,2023,2024,2025</t>
         </is>
       </c>
       <c r="D25" s="5" t="inlineStr">
         <is>
-          <t>%</t>
+          <t>years</t>
         </is>
       </c>
       <c r="E25" s="5" t="inlineStr"/>
       <c r="F25" s="5" t="inlineStr">
         <is>
-          <t>Write claimant rows above this % of the lowest AP [required]</t>
+          <t>Experience years used (comma list, 2-5 years) [required]</t>
         </is>
       </c>
       <c r="G25" s="6" t="n"/>
@@ -1835,7 +1827,7 @@
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
         <is>
-          <t>policy_limit</t>
+          <t>output_threshold_pct_min_ap</t>
         </is>
       </c>
       <c r="B26" s="5" t="inlineStr">
@@ -1843,16 +1835,20 @@
           <t>Data</t>
         </is>
       </c>
-      <c r="C26" s="6" t="n"/>
+      <c r="C26" s="6" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
       <c r="D26" s="5" t="inlineStr">
         <is>
-          <t>quote ccy</t>
+          <t>%</t>
         </is>
       </c>
       <c r="E26" s="5" t="inlineStr"/>
       <c r="F26" s="5" t="inlineStr">
         <is>
-          <t>Overall per-person policy limit (blank = none)</t>
+          <t>Write claimant rows above this % of the lowest AP [required]</t>
         </is>
       </c>
       <c r="G26" s="6" t="n"/>
@@ -1860,28 +1856,24 @@
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
         <is>
-          <t>outlier_method</t>
+          <t>policy_limit</t>
         </is>
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>Outliers</t>
-        </is>
-      </c>
-      <c r="C27" s="6" t="inlineStr">
-        <is>
-          <t>IQR</t>
-        </is>
-      </c>
-      <c r="D27" s="5" t="inlineStr"/>
-      <c r="E27" s="5" t="inlineStr">
-        <is>
-          <t>VALUE,IQR,NONE</t>
-        </is>
-      </c>
+          <t>Data</t>
+        </is>
+      </c>
+      <c r="C27" s="6" t="n"/>
+      <c r="D27" s="5" t="inlineStr">
+        <is>
+          <t>quote ccy</t>
+        </is>
+      </c>
+      <c r="E27" s="5" t="inlineStr"/>
       <c r="F27" s="5" t="inlineStr">
         <is>
-          <t>Outlier threshold rule [required]</t>
+          <t>Overall per-person policy limit (blank = none)</t>
         </is>
       </c>
       <c r="G27" s="6" t="n"/>
@@ -1889,7 +1881,7 @@
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
         <is>
-          <t>outlier_value</t>
+          <t>outlier_method</t>
         </is>
       </c>
       <c r="B28" s="5" t="inlineStr">
@@ -1897,16 +1889,20 @@
           <t>Outliers</t>
         </is>
       </c>
-      <c r="C28" s="6" t="n"/>
-      <c r="D28" s="5" t="inlineStr">
-        <is>
-          <t>quote ccy</t>
-        </is>
-      </c>
-      <c r="E28" s="5" t="inlineStr"/>
+      <c r="C28" s="6" t="inlineStr">
+        <is>
+          <t>IQR</t>
+        </is>
+      </c>
+      <c r="D28" s="5" t="inlineStr"/>
+      <c r="E28" s="5" t="inlineStr">
+        <is>
+          <t>VALUE,IQR,NONE</t>
+        </is>
+      </c>
       <c r="F28" s="5" t="inlineStr">
         <is>
-          <t>Threshold when outlier_method = VALUE</t>
+          <t>Outlier threshold rule [required]</t>
         </is>
       </c>
       <c r="G28" s="6" t="n"/>
@@ -1914,7 +1910,7 @@
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
         <is>
-          <t>iqr_multiplier</t>
+          <t>outlier_value</t>
         </is>
       </c>
       <c r="B29" s="5" t="inlineStr">
@@ -1922,20 +1918,16 @@
           <t>Outliers</t>
         </is>
       </c>
-      <c r="C29" s="6" t="inlineStr">
-        <is>
-          <t>1.5</t>
-        </is>
-      </c>
+      <c r="C29" s="6" t="n"/>
       <c r="D29" s="5" t="inlineStr">
         <is>
-          <t>x</t>
+          <t>quote ccy</t>
         </is>
       </c>
       <c r="E29" s="5" t="inlineStr"/>
       <c r="F29" s="5" t="inlineStr">
         <is>
-          <t>Multiplier when outlier_method = IQR</t>
+          <t>Threshold when outlier_method = VALUE</t>
         </is>
       </c>
       <c r="G29" s="6" t="n"/>
@@ -1943,28 +1935,28 @@
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
         <is>
-          <t>full_cred_n</t>
+          <t>iqr_multiplier</t>
         </is>
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t>Credibility</t>
+          <t>Outliers</t>
         </is>
       </c>
       <c r="C30" s="6" t="inlineStr">
         <is>
-          <t>64</t>
+          <t>1.5</t>
         </is>
       </c>
       <c r="D30" s="5" t="inlineStr">
         <is>
-          <t>claims</t>
+          <t>x</t>
         </is>
       </c>
       <c r="E30" s="5" t="inlineStr"/>
       <c r="F30" s="5" t="inlineStr">
         <is>
-          <t>Claims for full credibility (workshop default 64) [required]</t>
+          <t>Multiplier when outlier_method = IQR</t>
         </is>
       </c>
       <c r="G30" s="6" t="n"/>
@@ -1972,7 +1964,7 @@
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
-          <t>complement_source</t>
+          <t>full_cred_n</t>
         </is>
       </c>
       <c r="B31" s="5" t="inlineStr">
@@ -1982,18 +1974,18 @@
       </c>
       <c r="C31" s="6" t="inlineStr">
         <is>
-          <t>STOCHASTIC</t>
-        </is>
-      </c>
-      <c r="D31" s="5" t="inlineStr"/>
-      <c r="E31" s="5" t="inlineStr">
-        <is>
-          <t>STOCHASTIC,BENCHMARK,EXPIRING</t>
-        </is>
-      </c>
+          <t>64</t>
+        </is>
+      </c>
+      <c r="D31" s="5" t="inlineStr">
+        <is>
+          <t>claims</t>
+        </is>
+      </c>
+      <c r="E31" s="5" t="inlineStr"/>
       <c r="F31" s="5" t="inlineStr">
         <is>
-          <t>Credibility complement [required]</t>
+          <t>Claims for full credibility (workshop default 64) [required]</t>
         </is>
       </c>
       <c r="G31" s="6" t="n"/>
@@ -2001,7 +1993,7 @@
     <row r="32">
       <c r="A32" s="5" t="inlineStr">
         <is>
-          <t>benchmark_rate</t>
+          <t>complement_source</t>
         </is>
       </c>
       <c r="B32" s="5" t="inlineStr">
@@ -2009,16 +2001,20 @@
           <t>Credibility</t>
         </is>
       </c>
-      <c r="C32" s="6" t="n"/>
-      <c r="D32" s="5" t="inlineStr">
-        <is>
-          <t>quote ccy pppy</t>
-        </is>
-      </c>
-      <c r="E32" s="5" t="inlineStr"/>
+      <c r="C32" s="6" t="inlineStr">
+        <is>
+          <t>STOCHASTIC</t>
+        </is>
+      </c>
+      <c r="D32" s="5" t="inlineStr"/>
+      <c r="E32" s="5" t="inlineStr">
+        <is>
+          <t>STOCHASTIC,BENCHMARK,EXPIRING</t>
+        </is>
+      </c>
       <c r="F32" s="5" t="inlineStr">
         <is>
-          <t>When complement_source = BENCHMARK</t>
+          <t>Credibility complement [required]</t>
         </is>
       </c>
       <c r="G32" s="6" t="n"/>
@@ -2026,45 +2022,37 @@
     <row r="33">
       <c r="A33" s="5" t="inlineStr">
         <is>
-          <t>incidence_adj</t>
+          <t>benchmark_rate</t>
         </is>
       </c>
       <c r="B33" s="5" t="inlineStr">
         <is>
-          <t>Incidence</t>
-        </is>
-      </c>
-      <c r="C33" s="6" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>Credibility</t>
+        </is>
+      </c>
+      <c r="C33" s="6" t="n"/>
       <c r="D33" s="5" t="inlineStr">
         <is>
-          <t>x</t>
+          <t>quote ccy pppy</t>
         </is>
       </c>
       <c r="E33" s="5" t="inlineStr"/>
       <c r="F33" s="5" t="inlineStr">
         <is>
-          <t>Overall incidence adjustment (1 = none); justify [required]</t>
-        </is>
-      </c>
-      <c r="G33" s="6" t="inlineStr">
-        <is>
-          <t>No explained trend outside the trend assumption</t>
-        </is>
-      </c>
+          <t>When complement_source = BENCHMARK</t>
+        </is>
+      </c>
+      <c r="G33" s="6" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="5" t="inlineStr">
         <is>
-          <t>qs_cedant_retention_pct</t>
+          <t>incidence_adj</t>
         </is>
       </c>
       <c r="B34" s="5" t="inlineStr">
         <is>
-          <t>QS</t>
+          <t>Incidence</t>
         </is>
       </c>
       <c r="C34" s="6" t="inlineStr">
@@ -2074,42 +2062,46 @@
       </c>
       <c r="D34" s="5" t="inlineStr">
         <is>
-          <t>%</t>
+          <t>x</t>
         </is>
       </c>
       <c r="E34" s="5" t="inlineStr"/>
       <c r="F34" s="5" t="inlineStr">
         <is>
-          <t>Cedant retention under an existing QS (1 = no QS) [required]</t>
-        </is>
-      </c>
-      <c r="G34" s="6" t="n"/>
+          <t>Overall incidence adjustment (1 = none); justify [required]</t>
+        </is>
+      </c>
+      <c r="G34" s="6" t="inlineStr">
+        <is>
+          <t>No explained trend outside the trend assumption</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="5" t="inlineStr">
         <is>
-          <t>evaluate_mode</t>
+          <t>qs_cedant_retention_pct</t>
         </is>
       </c>
       <c r="B35" s="5" t="inlineStr">
         <is>
-          <t>Programme</t>
+          <t>QS</t>
         </is>
       </c>
       <c r="C35" s="6" t="inlineStr">
         <is>
-          <t>STANDALONE</t>
-        </is>
-      </c>
-      <c r="D35" s="5" t="inlineStr"/>
-      <c r="E35" s="5" t="inlineStr">
-        <is>
-          <t>STANDALONE,PROGRAMME</t>
-        </is>
-      </c>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D35" s="5" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E35" s="5" t="inlineStr"/>
       <c r="F35" s="5" t="inlineStr">
         <is>
-          <t>Options standalone, or stacked per Programme [required]</t>
+          <t>Cedant retention under an existing QS (1 = no QS) [required]</t>
         </is>
       </c>
       <c r="G35" s="6" t="n"/>
@@ -2117,28 +2109,28 @@
     <row r="36">
       <c r="A36" s="5" t="inlineStr">
         <is>
-          <t>iterations</t>
+          <t>evaluate_mode</t>
         </is>
       </c>
       <c r="B36" s="5" t="inlineStr">
         <is>
-          <t>Stochastic</t>
+          <t>Programme</t>
         </is>
       </c>
       <c r="C36" s="6" t="inlineStr">
         <is>
-          <t>10000</t>
-        </is>
-      </c>
-      <c r="D36" s="5" t="inlineStr">
-        <is>
-          <t>n</t>
-        </is>
-      </c>
-      <c r="E36" s="5" t="inlineStr"/>
+          <t>STANDALONE</t>
+        </is>
+      </c>
+      <c r="D36" s="5" t="inlineStr"/>
+      <c r="E36" s="5" t="inlineStr">
+        <is>
+          <t>STANDALONE,PROGRAMME</t>
+        </is>
+      </c>
       <c r="F36" s="5" t="inlineStr">
         <is>
-          <t>Simulation iterations [required]</t>
+          <t>Options standalone, or stacked per Programme [required]</t>
         </is>
       </c>
       <c r="G36" s="6" t="n"/>
@@ -2146,7 +2138,7 @@
     <row r="37">
       <c r="A37" s="5" t="inlineStr">
         <is>
-          <t>seed</t>
+          <t>iterations</t>
         </is>
       </c>
       <c r="B37" s="5" t="inlineStr">
@@ -2156,14 +2148,18 @@
       </c>
       <c r="C37" s="6" t="inlineStr">
         <is>
-          <t>12345</t>
-        </is>
-      </c>
-      <c r="D37" s="5" t="inlineStr"/>
+          <t>10000</t>
+        </is>
+      </c>
+      <c r="D37" s="5" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
       <c r="E37" s="5" t="inlineStr"/>
       <c r="F37" s="5" t="inlineStr">
         <is>
-          <t>Random seed (recorded in the run log) [required]</t>
+          <t>Simulation iterations [required]</t>
         </is>
       </c>
       <c r="G37" s="6" t="n"/>
@@ -2171,7 +2167,7 @@
     <row r="38">
       <c r="A38" s="5" t="inlineStr">
         <is>
-          <t>fit_cutoff</t>
+          <t>seed</t>
         </is>
       </c>
       <c r="B38" s="5" t="inlineStr">
@@ -2179,16 +2175,16 @@
           <t>Stochastic</t>
         </is>
       </c>
-      <c r="C38" s="6" t="n"/>
-      <c r="D38" s="5" t="inlineStr">
-        <is>
-          <t>quote ccy</t>
-        </is>
-      </c>
+      <c r="C38" s="6" t="inlineStr">
+        <is>
+          <t>12345</t>
+        </is>
+      </c>
+      <c r="D38" s="5" t="inlineStr"/>
       <c r="E38" s="5" t="inlineStr"/>
       <c r="F38" s="5" t="inlineStr">
         <is>
-          <t>Severity fitting cut-off (blank = AP)</t>
+          <t>Random seed (recorded in the run log) [required]</t>
         </is>
       </c>
       <c r="G38" s="6" t="n"/>
@@ -2196,7 +2192,7 @@
     <row r="39">
       <c r="A39" s="5" t="inlineStr">
         <is>
-          <t>fit_candidates</t>
+          <t>fit_cutoff</t>
         </is>
       </c>
       <c r="B39" s="5" t="inlineStr">
@@ -2204,16 +2200,16 @@
           <t>Stochastic</t>
         </is>
       </c>
-      <c r="C39" s="6" t="inlineStr">
-        <is>
-          <t>LOGNORMAL,GAMMA,WEIBULL,PARETO,GPD</t>
-        </is>
-      </c>
-      <c r="D39" s="5" t="inlineStr"/>
+      <c r="C39" s="6" t="n"/>
+      <c r="D39" s="5" t="inlineStr">
+        <is>
+          <t>quote ccy</t>
+        </is>
+      </c>
       <c r="E39" s="5" t="inlineStr"/>
       <c r="F39" s="5" t="inlineStr">
         <is>
-          <t>Candidate severity distributions [required]</t>
+          <t>Severity fitting cut-off (blank = AP)</t>
         </is>
       </c>
       <c r="G39" s="6" t="n"/>
@@ -2221,7 +2217,7 @@
     <row r="40">
       <c r="A40" s="5" t="inlineStr">
         <is>
-          <t>fit_selected</t>
+          <t>fit_candidates</t>
         </is>
       </c>
       <c r="B40" s="5" t="inlineStr">
@@ -2229,16 +2225,16 @@
           <t>Stochastic</t>
         </is>
       </c>
-      <c r="C40" s="6" t="n"/>
+      <c r="C40" s="6" t="inlineStr">
+        <is>
+          <t>LOGNORMAL,GAMMA,WEIBULL,PARETO,GPD</t>
+        </is>
+      </c>
       <c r="D40" s="5" t="inlineStr"/>
-      <c r="E40" s="5" t="inlineStr">
-        <is>
-          <t>LOGNORMAL,GAMMA,WEIBULL,PARETO,GPD</t>
-        </is>
-      </c>
+      <c r="E40" s="5" t="inlineStr"/>
       <c r="F40" s="5" t="inlineStr">
         <is>
-          <t>Severity distribution used by the simulation (blank = lowest AIC in stage 04a); justify an override</t>
+          <t>Candidate severity distributions [required]</t>
         </is>
       </c>
       <c r="G40" s="6" t="n"/>
@@ -2246,7 +2242,7 @@
     <row r="41">
       <c r="A41" s="5" t="inlineStr">
         <is>
-          <t>severity_source</t>
+          <t>fit_selected</t>
         </is>
       </c>
       <c r="B41" s="5" t="inlineStr">
@@ -2254,20 +2250,16 @@
           <t>Stochastic</t>
         </is>
       </c>
-      <c r="C41" s="6" t="inlineStr">
-        <is>
-          <t>PYTHON</t>
-        </is>
-      </c>
+      <c r="C41" s="6" t="n"/>
       <c r="D41" s="5" t="inlineStr"/>
       <c r="E41" s="5" t="inlineStr">
         <is>
-          <t>PYTHON,NATIVE</t>
+          <t>LOGNORMAL,GAMMA,WEIBULL,PARETO,GPD</t>
         </is>
       </c>
       <c r="F41" s="5" t="inlineStr">
         <is>
-          <t>PYTHON: distribution selected in 04a_fit_severity (Python tool); NATIVE: Pareto fitted in stage 04 (no Python) [required]</t>
+          <t>Severity distribution used by the simulation (blank = lowest AIC in stage 04a); justify an override</t>
         </is>
       </c>
       <c r="G41" s="6" t="n"/>
@@ -2275,7 +2267,7 @@
     <row r="42">
       <c r="A42" s="5" t="inlineStr">
         <is>
-          <t>freq_model</t>
+          <t>severity_source</t>
         </is>
       </c>
       <c r="B42" s="5" t="inlineStr">
@@ -2285,18 +2277,18 @@
       </c>
       <c r="C42" s="6" t="inlineStr">
         <is>
-          <t>POISSON</t>
+          <t>PYTHON</t>
         </is>
       </c>
       <c r="D42" s="5" t="inlineStr"/>
       <c r="E42" s="5" t="inlineStr">
         <is>
-          <t>POISSON,NEGBIN</t>
+          <t>PYTHON,NATIVE</t>
         </is>
       </c>
       <c r="F42" s="5" t="inlineStr">
         <is>
-          <t>Frequency distribution [required]</t>
+          <t>PYTHON: distribution selected in 04a_fit_severity (Python tool); NATIVE: Pareto fitted in stage 04 (no Python) [required]</t>
         </is>
       </c>
       <c r="G42" s="6" t="n"/>
@@ -2304,7 +2296,7 @@
     <row r="43">
       <c r="A43" s="5" t="inlineStr">
         <is>
-          <t>ev_freq_source</t>
+          <t>freq_model</t>
         </is>
       </c>
       <c r="B43" s="5" t="inlineStr">
@@ -2314,18 +2306,18 @@
       </c>
       <c r="C43" s="6" t="inlineStr">
         <is>
-          <t>BOTH</t>
+          <t>POISSON</t>
         </is>
       </c>
       <c r="D43" s="5" t="inlineStr"/>
       <c r="E43" s="5" t="inlineStr">
         <is>
-          <t>EXPERIENCE,SCENARIOS,BOTH</t>
+          <t>POISSON,NEGBIN</t>
         </is>
       </c>
       <c r="F43" s="5" t="inlineStr">
         <is>
-          <t>Per-event simulation: historical events, EvScenarios (with a return period), or both [required]</t>
+          <t>Frequency distribution [required]</t>
         </is>
       </c>
       <c r="G43" s="6" t="n"/>
@@ -2333,7 +2325,7 @@
     <row r="44">
       <c r="A44" s="5" t="inlineStr">
         <is>
-          <t>sl_attritional_threshold</t>
+          <t>ev_freq_source</t>
         </is>
       </c>
       <c r="B44" s="5" t="inlineStr">
@@ -2343,18 +2335,18 @@
       </c>
       <c r="C44" s="6" t="inlineStr">
         <is>
-          <t>100000</t>
-        </is>
-      </c>
-      <c r="D44" s="5" t="inlineStr">
-        <is>
-          <t>quote ccy</t>
-        </is>
-      </c>
-      <c r="E44" s="5" t="inlineStr"/>
+          <t>BOTH</t>
+        </is>
+      </c>
+      <c r="D44" s="5" t="inlineStr"/>
+      <c r="E44" s="5" t="inlineStr">
+        <is>
+          <t>EXPERIENCE,SCENARIOS,BOTH</t>
+        </is>
+      </c>
       <c r="F44" s="5" t="inlineStr">
         <is>
-          <t>Stop loss: attritional / large split [required]</t>
+          <t>Per-event simulation: historical events, EvScenarios (with a return period), or both [required]</t>
         </is>
       </c>
       <c r="G44" s="6" t="n"/>
@@ -2362,7 +2354,7 @@
     <row r="45">
       <c r="A45" s="5" t="inlineStr">
         <is>
-          <t>sl_cov_floor</t>
+          <t>sl_attritional_threshold</t>
         </is>
       </c>
       <c r="B45" s="5" t="inlineStr">
@@ -2372,14 +2364,18 @@
       </c>
       <c r="C45" s="6" t="inlineStr">
         <is>
-          <t>0.05</t>
-        </is>
-      </c>
-      <c r="D45" s="5" t="inlineStr"/>
+          <t>100000</t>
+        </is>
+      </c>
+      <c r="D45" s="5" t="inlineStr">
+        <is>
+          <t>quote ccy</t>
+        </is>
+      </c>
       <c r="E45" s="5" t="inlineStr"/>
       <c r="F45" s="5" t="inlineStr">
         <is>
-          <t>Stop loss: minimum CoV of the attritional cost per life [required]</t>
+          <t>Stop loss: attritional / large split [required]</t>
         </is>
       </c>
       <c r="G45" s="6" t="n"/>
@@ -2387,7 +2383,7 @@
     <row r="46">
       <c r="A46" s="5" t="inlineStr">
         <is>
-          <t>sl_attritional_dist</t>
+          <t>sl_cov_floor</t>
         </is>
       </c>
       <c r="B46" s="5" t="inlineStr">
@@ -2397,18 +2393,14 @@
       </c>
       <c r="C46" s="6" t="inlineStr">
         <is>
-          <t>LOGNORMAL</t>
+          <t>0.05</t>
         </is>
       </c>
       <c r="D46" s="5" t="inlineStr"/>
-      <c r="E46" s="5" t="inlineStr">
-        <is>
-          <t>LOGNORMAL,NORMAL</t>
-        </is>
-      </c>
+      <c r="E46" s="5" t="inlineStr"/>
       <c r="F46" s="5" t="inlineStr">
         <is>
-          <t>Stop loss: distribution of the attritional cost per life [required]</t>
+          <t>Stop loss: minimum CoV of the attritional cost per life [required]</t>
         </is>
       </c>
       <c r="G46" s="6" t="n"/>
@@ -2416,24 +2408,28 @@
     <row r="47">
       <c r="A47" s="5" t="inlineStr">
         <is>
-          <t>net_claims_budget</t>
+          <t>sl_attritional_dist</t>
         </is>
       </c>
       <c r="B47" s="5" t="inlineStr">
         <is>
-          <t>Cedant impact</t>
-        </is>
-      </c>
-      <c r="C47" s="6" t="n"/>
-      <c r="D47" s="5" t="inlineStr">
-        <is>
-          <t>quote ccy</t>
-        </is>
-      </c>
-      <c r="E47" s="5" t="inlineStr"/>
+          <t>Stochastic</t>
+        </is>
+      </c>
+      <c r="C47" s="6" t="inlineStr">
+        <is>
+          <t>LOGNORMAL</t>
+        </is>
+      </c>
+      <c r="D47" s="5" t="inlineStr"/>
+      <c r="E47" s="5" t="inlineStr">
+        <is>
+          <t>LOGNORMAL,NORMAL</t>
+        </is>
+      </c>
       <c r="F47" s="5" t="inlineStr">
         <is>
-          <t>Blank = best-estimate gross claims</t>
+          <t>Stop loss: distribution of the attritional cost per life [required]</t>
         </is>
       </c>
       <c r="G47" s="6" t="n"/>
@@ -2441,7 +2437,7 @@
     <row r="48">
       <c r="A48" s="5" t="inlineStr">
         <is>
-          <t>reference_lives</t>
+          <t>net_claims_budget</t>
         </is>
       </c>
       <c r="B48" s="5" t="inlineStr">
@@ -2449,16 +2445,16 @@
           <t>Cedant impact</t>
         </is>
       </c>
-      <c r="C48" s="6" t="inlineStr"/>
+      <c r="C48" s="6" t="n"/>
       <c r="D48" s="5" t="inlineStr">
         <is>
-          <t>lives</t>
+          <t>quote ccy</t>
         </is>
       </c>
       <c r="E48" s="5" t="inlineStr"/>
       <c r="F48" s="5" t="inlineStr">
         <is>
-          <t>Blank = expected lives for the quote year</t>
+          <t>Blank = best-estimate gross claims</t>
         </is>
       </c>
       <c r="G48" s="6" t="n"/>
@@ -2466,7 +2462,7 @@
     <row r="49">
       <c r="A49" s="5" t="inlineStr">
         <is>
-          <t>return_periods</t>
+          <t>reference_lives</t>
         </is>
       </c>
       <c r="B49" s="5" t="inlineStr">
@@ -2474,20 +2470,16 @@
           <t>Cedant impact</t>
         </is>
       </c>
-      <c r="C49" s="6" t="inlineStr">
-        <is>
-          <t>5,50,250</t>
-        </is>
-      </c>
+      <c r="C49" s="6" t="inlineStr"/>
       <c r="D49" s="5" t="inlineStr">
         <is>
-          <t>years</t>
+          <t>lives</t>
         </is>
       </c>
       <c r="E49" s="5" t="inlineStr"/>
       <c r="F49" s="5" t="inlineStr">
         <is>
-          <t>Return periods shown in Exhibit C2 [required]</t>
+          <t>Blank = expected lives for the quote year</t>
         </is>
       </c>
       <c r="G49" s="6" t="n"/>
@@ -2495,31 +2487,60 @@
     <row r="50">
       <c r="A50" s="5" t="inlineStr">
         <is>
+          <t>return_periods</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="inlineStr">
+        <is>
+          <t>Cedant impact</t>
+        </is>
+      </c>
+      <c r="C50" s="6" t="inlineStr">
+        <is>
+          <t>5,50,250</t>
+        </is>
+      </c>
+      <c r="D50" s="5" t="inlineStr">
+        <is>
+          <t>years</t>
+        </is>
+      </c>
+      <c r="E50" s="5" t="inlineStr"/>
+      <c r="F50" s="5" t="inlineStr">
+        <is>
+          <t>Return periods shown in Exhibit C2 [required]</t>
+        </is>
+      </c>
+      <c r="G50" s="6" t="n"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
           <t>currency_display</t>
         </is>
       </c>
-      <c r="B50" s="5" t="inlineStr">
+      <c r="B51" s="5" t="inlineStr">
         <is>
           <t>Cedant impact</t>
         </is>
       </c>
-      <c r="C50" s="6" t="inlineStr">
+      <c r="C51" s="6" t="inlineStr">
         <is>
           <t>QUOTE</t>
         </is>
       </c>
-      <c r="D50" s="5" t="inlineStr"/>
-      <c r="E50" s="5" t="inlineStr">
+      <c r="D51" s="5" t="inlineStr"/>
+      <c r="E51" s="5" t="inlineStr">
         <is>
           <t>QUOTE,USD</t>
         </is>
       </c>
-      <c r="F50" s="5" t="inlineStr">
+      <c r="F51" s="5" t="inlineStr">
         <is>
           <t>Currency of the client exhibits [required]</t>
         </is>
       </c>
-      <c r="G50" s="6" t="n"/>
+      <c r="G51" s="6" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -2532,40 +2553,40 @@
     <dataValidation sqref="C15" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"GROSS,GROSSNET,NET"</formula1>
     </dataValidation>
-    <dataValidation sqref="C18" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="C19" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"RA,LO"</formula1>
     </dataValidation>
-    <dataValidation sqref="C19" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="C20" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"INCURRED,PAID"</formula1>
     </dataValidation>
-    <dataValidation sqref="C21" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="C22" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"POLICY_YEAR,TREATY_YEAR"</formula1>
     </dataValidation>
-    <dataValidation sqref="C27" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="C28" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"VALUE,IQR,NONE"</formula1>
     </dataValidation>
-    <dataValidation sqref="C31" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="C32" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"STOCHASTIC,BENCHMARK,EXPIRING"</formula1>
     </dataValidation>
-    <dataValidation sqref="C35" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="C36" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"STANDALONE,PROGRAMME"</formula1>
     </dataValidation>
-    <dataValidation sqref="C40" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="C41" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"LOGNORMAL,GAMMA,WEIBULL,PARETO,GPD"</formula1>
     </dataValidation>
-    <dataValidation sqref="C41" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="C42" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"PYTHON,NATIVE"</formula1>
     </dataValidation>
-    <dataValidation sqref="C42" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="C43" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"POISSON,NEGBIN"</formula1>
     </dataValidation>
-    <dataValidation sqref="C43" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="C44" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"EXPERIENCE,SCENARIOS,BOTH"</formula1>
     </dataValidation>
-    <dataValidation sqref="C46" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="C47" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"LOGNORMAL,NORMAL"</formula1>
     </dataValidation>
-    <dataValidation sqref="C50" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="C51" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"QUOTE,USD"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>